<commit_message>
Daily NSE scan: 2026-09-04
</commit_message>
<xml_diff>
--- a/output/2026-09-04/enriched_analysis.xlsx
+++ b/output/2026-09-04/enriched_analysis.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gandhar Oil Refinery (India) Limited</t>
+          <t>GANDHAR OIL REFINERY (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>THANGAMAYIL JEWELLERY LIMITED</t>
+          <t>THANGAMAIYL JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PNGS Reva Diamond Jewellery Limited</t>
+          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Ganesh Consumer Products Limited</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gandhar Oil Refinery (India) Limited</t>
+          <t>GANDHAR OIL REFINERY (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>THANGAMAYIL JEWELLERY LIMITED</t>
+          <t>THANGAMAIYL JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -5462,7 +5462,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PNGS Reva Diamond Jewellery Limited</t>
+          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -6372,7 +6372,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Ganesh Consumer Products Limited</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C35" t="n">

</xml_diff>